<commit_message>
Nhat: update w1 report
</commit_message>
<xml_diff>
--- a/docs/25410104_NguyenMinhNhat_25410034_LeQuangHoaiDuc - Kế hoạch thực hiện đồ án, chuyên đề.xlsx
+++ b/docs/25410104_NguyenMinhNhat_25410034_LeQuangHoaiDuc - Kế hoạch thực hiện đồ án, chuyên đề.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{097A257F-78F8-47A5-A0FA-0EA42C44EC57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{377EB757-6E1F-47DD-A156-9021669DBD54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,9 +27,6 @@
   </si>
   <si>
     <t>PHÂN BỐ THỜI GIAN THỰC HIỆN</t>
-  </si>
-  <si>
-    <t>Kiểm tra và sửa lỗi</t>
   </si>
   <si>
     <r>
@@ -56,18 +53,6 @@
   </si>
   <si>
     <t>Mức độ hoàn thành</t>
-  </si>
-  <si>
-    <t>Thực nghiệm và đánh giá, khảo sát các tính năng của hệ thống.</t>
-  </si>
-  <si>
-    <t>Viết báo cáo đồ án môn học x</t>
-  </si>
-  <si>
-    <t>Báo cáo đồ án môn học x</t>
-  </si>
-  <si>
-    <t>Báo cáo giữa kỳ</t>
   </si>
   <si>
     <r>
@@ -160,39 +145,91 @@
   </si>
   <si>
     <t>1
-(22/7 - 29/7)</t>
+(15-7-21/7)</t>
   </si>
   <si>
     <t>2
-(29/7 - 5/8)</t>
+(22/7 - 28/7)</t>
   </si>
   <si>
     <t>3
-(5/8 - 12/8)</t>
+(29/7 - 4/8)</t>
   </si>
   <si>
     <t>4
-(12/8 - 19/8)</t>
+(5/8 - 11/8)</t>
   </si>
   <si>
     <t>5
-(19/8 - 26/8)</t>
+(12/8 - 18/8)</t>
   </si>
   <si>
     <t>6
-(26/8 - 2/9)</t>
+(19/8 - 25/8)</t>
   </si>
   <si>
     <t>7
-(2/9 - 9/9)</t>
+(26/8 - 1/9)</t>
   </si>
   <si>
     <t>8
-(9/9 - 16/9)</t>
+(2/9 - 8/9)</t>
   </si>
   <si>
     <t>9
-(16/9 - 23/9)</t>
+(9/9 - 15/9)</t>
+  </si>
+  <si>
+    <t>10
+(16/9 - 22/9)</t>
+  </si>
+  <si>
+    <t>Báo cáo đồ án môn học</t>
+  </si>
+  <si>
+    <t>22/7/2026</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Nhật</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>: Hoàn thành, tạo file MD cho 2 phần được giao trong source code</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Nhật</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>: research,  khảo sát các hệ thống ALPR/nhận diện phương tiện tương tự (mã nguồn mở, thương mại, trong nước, dataset tham chiếu), và tổng hợp quy định biển số xe Việt Nam (căn cứ pháp lý, cấu trúc ký tự, số lượng/bố cục biển theo loại xe, chất liệu, bảng màu biển)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -568,7 +605,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -623,9 +660,6 @@
     </xf>
     <xf numFmtId="49" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
@@ -718,9 +752,6 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -772,6 +803,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1101,7 +1141,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -1119,13 +1159,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="52.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="71" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
+      <c r="A1" s="69" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
       <c r="F1" s="14"/>
       <c r="G1" s="14"/>
       <c r="H1" s="14"/>
@@ -1134,13 +1174,13 @@
       <c r="K1" s="5"/>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="73" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="74"/>
-      <c r="D2" s="74"/>
-      <c r="E2" s="74"/>
+      <c r="A2" s="71" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
@@ -1149,11 +1189,11 @@
       <c r="K2" s="6"/>
     </row>
     <row r="3" spans="1:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="73"/>
-      <c r="B3" s="74"/>
-      <c r="C3" s="74"/>
-      <c r="D3" s="74"/>
-      <c r="E3" s="74"/>
+      <c r="A3" s="71"/>
+      <c r="B3" s="72"/>
+      <c r="C3" s="72"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="72"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -1162,13 +1202,13 @@
       <c r="K3" s="6"/>
     </row>
     <row r="4" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="73" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="74"/>
-      <c r="C4" s="74"/>
-      <c r="D4" s="74"/>
-      <c r="E4" s="74"/>
+      <c r="A4" s="71" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="72"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="72"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
@@ -1177,11 +1217,11 @@
       <c r="K4" s="2"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="73"/>
-      <c r="B5" s="74"/>
-      <c r="C5" s="74"/>
-      <c r="D5" s="74"/>
-      <c r="E5" s="74"/>
+      <c r="A5" s="71"/>
+      <c r="B5" s="72"/>
+      <c r="C5" s="72"/>
+      <c r="D5" s="72"/>
+      <c r="E5" s="72"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -1190,11 +1230,11 @@
       <c r="K5" s="2"/>
     </row>
     <row r="6" spans="1:11" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="73"/>
-      <c r="B6" s="74"/>
-      <c r="C6" s="74"/>
-      <c r="D6" s="74"/>
-      <c r="E6" s="74"/>
+      <c r="A6" s="71"/>
+      <c r="B6" s="72"/>
+      <c r="C6" s="72"/>
+      <c r="D6" s="72"/>
+      <c r="E6" s="72"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -1203,266 +1243,279 @@
       <c r="K6" s="2"/>
     </row>
     <row r="7" spans="1:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="75" t="s">
+      <c r="A7" s="73" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="76"/>
-      <c r="C7" s="76"/>
-      <c r="D7" s="76"/>
-      <c r="E7" s="76"/>
-      <c r="F7" s="53"/>
-      <c r="G7" s="53"/>
-      <c r="H7" s="53"/>
-      <c r="I7" s="53"/>
+      <c r="B7" s="74"/>
+      <c r="C7" s="74"/>
+      <c r="D7" s="74"/>
+      <c r="E7" s="74"/>
+      <c r="F7" s="52"/>
+      <c r="G7" s="52"/>
+      <c r="H7" s="52"/>
+      <c r="I7" s="52"/>
       <c r="J7" s="16"/>
     </row>
-    <row r="8" spans="1:11" s="4" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="54"/>
+    <row r="8" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="53"/>
       <c r="B8" s="12" t="s">
         <v>0</v>
       </c>
       <c r="C8" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="E8" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="F8" s="51"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="31"/>
-      <c r="I8" s="35"/>
-      <c r="J8" s="37"/>
-      <c r="K8" s="36"/>
-    </row>
-    <row r="9" spans="1:11" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="70"/>
-      <c r="B9" s="10" t="s">
+      <c r="E8" s="25" t="s">
+        <v>5</v>
+      </c>
+      <c r="F8" s="50"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="34"/>
+      <c r="J8" s="36"/>
+      <c r="K8" s="35"/>
+    </row>
+    <row r="9" spans="1:11" s="4" customFormat="1" ht="78" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="53"/>
+      <c r="B9" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="54" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="54" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="75"/>
+      <c r="G9" s="75"/>
+      <c r="H9" s="76"/>
+      <c r="I9" s="34"/>
+      <c r="J9" s="77"/>
+      <c r="K9" s="75"/>
+    </row>
+    <row r="10" spans="1:11" ht="78" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="68"/>
+      <c r="B10" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="17"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="11"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="38"/>
+      <c r="J10" s="37"/>
+    </row>
+    <row r="11" spans="1:11" ht="78" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="68"/>
+      <c r="B11" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="54"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="60"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="33"/>
+      <c r="I11" s="39"/>
+      <c r="J11" s="39"/>
+      <c r="K11" s="31"/>
+    </row>
+    <row r="12" spans="1:11" ht="78" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="68"/>
+      <c r="B12" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="58"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="40"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="31"/>
+    </row>
+    <row r="13" spans="1:11" ht="78" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="68"/>
+      <c r="B13" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="55"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="56"/>
+      <c r="F13" s="51"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="41"/>
+      <c r="I13" s="42"/>
+      <c r="J13" s="42"/>
+      <c r="K13" s="31"/>
+    </row>
+    <row r="14" spans="1:11" ht="78" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="68"/>
+      <c r="B14" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="17"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="11"/>
-      <c r="H9" s="33"/>
-      <c r="I9" s="39"/>
-      <c r="J9" s="38"/>
-    </row>
-    <row r="10" spans="1:11" ht="122.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="70"/>
-      <c r="B10" s="19" t="s">
+      <c r="C14" s="58"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="62"/>
+      <c r="F14" s="49"/>
+      <c r="G14" s="38"/>
+      <c r="H14" s="43"/>
+      <c r="I14" s="42"/>
+      <c r="J14" s="42"/>
+      <c r="K14" s="31"/>
+    </row>
+    <row r="15" spans="1:11" ht="78" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="68"/>
+      <c r="B15" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="55"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="62"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="29"/>
-      <c r="H10" s="34"/>
-      <c r="I10" s="40"/>
-      <c r="J10" s="40"/>
-      <c r="K10" s="32"/>
-    </row>
-    <row r="11" spans="1:11" ht="77.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="70"/>
-      <c r="B11" s="10" t="s">
+      <c r="C15" s="63"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="56"/>
+      <c r="F15" s="49"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="45"/>
+      <c r="I15" s="42"/>
+      <c r="J15" s="42"/>
+      <c r="K15" s="31"/>
+    </row>
+    <row r="16" spans="1:11" ht="78" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="68"/>
+      <c r="B16" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="60"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="63"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="29"/>
-      <c r="H11" s="29"/>
-      <c r="I11" s="41"/>
-      <c r="J11" s="20"/>
-      <c r="K11" s="32"/>
-    </row>
-    <row r="12" spans="1:11" ht="63.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="70"/>
-      <c r="B12" s="19" t="s">
+      <c r="C16" s="58"/>
+      <c r="D16" s="58"/>
+      <c r="E16" s="57"/>
+      <c r="F16" s="49"/>
+      <c r="G16" s="44"/>
+      <c r="H16" s="45"/>
+      <c r="I16" s="42"/>
+      <c r="J16" s="42"/>
+      <c r="K16" s="31"/>
+    </row>
+    <row r="17" spans="1:11" ht="78" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="68"/>
+      <c r="B17" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="56"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="58"/>
-      <c r="F12" s="52"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="42"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="43"/>
-      <c r="K12" s="32"/>
-    </row>
-    <row r="13" spans="1:11" ht="62.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="70"/>
-      <c r="B13" s="18" t="s">
+      <c r="C17" s="63"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="56"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="46"/>
+      <c r="H17" s="47"/>
+      <c r="I17" s="48"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="31"/>
+    </row>
+    <row r="18" spans="1:11" ht="78" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="68"/>
+      <c r="B18" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="57" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="23"/>
-      <c r="E13" s="64"/>
-      <c r="F13" s="50"/>
-      <c r="G13" s="39"/>
-      <c r="H13" s="44"/>
-      <c r="I13" s="43"/>
-      <c r="J13" s="43"/>
-      <c r="K13" s="32"/>
-    </row>
-    <row r="14" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="70"/>
-      <c r="B14" s="19" t="s">
+      <c r="C18" s="58"/>
+      <c r="D18" s="58"/>
+      <c r="E18" s="57"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="46"/>
+      <c r="H18" s="47"/>
+      <c r="I18" s="48"/>
+      <c r="J18" s="20"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="68"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="65"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="58"/>
-      <c r="F14" s="50"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="43"/>
-      <c r="J14" s="43"/>
-      <c r="K14" s="32"/>
-    </row>
-    <row r="15" spans="1:11" ht="90.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="70"/>
-      <c r="B15" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="C15" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="25"/>
-      <c r="E15" s="59"/>
-      <c r="F15" s="50"/>
-      <c r="G15" s="45"/>
-      <c r="H15" s="46"/>
-      <c r="I15" s="43"/>
-      <c r="J15" s="43"/>
-      <c r="K15" s="32"/>
-    </row>
-    <row r="16" spans="1:11" ht="58.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="70"/>
-      <c r="B16" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D16" s="23"/>
-      <c r="E16" s="61"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="47"/>
-      <c r="H16" s="48"/>
-      <c r="I16" s="49"/>
-      <c r="J16" s="20"/>
-      <c r="K16" s="32"/>
-    </row>
-    <row r="17" spans="1:10" ht="58.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="70"/>
-      <c r="B17" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D17" s="25"/>
-      <c r="E17" s="61"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="47"/>
-      <c r="H17" s="48"/>
-      <c r="I17" s="49"/>
-      <c r="J17" s="20"/>
-    </row>
-    <row r="18" spans="1:10" ht="58.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="70"/>
-      <c r="B18" s="19"/>
-      <c r="C18" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="25"/>
-      <c r="E18" s="61"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="47"/>
-      <c r="H18" s="48"/>
-      <c r="I18" s="49"/>
-      <c r="J18" s="20"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="3"/>
-      <c r="C19" s="8"/>
-      <c r="E19" s="27"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D19" s="24"/>
+      <c r="E19" s="59"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="46"/>
+      <c r="H19" s="47"/>
+      <c r="I19" s="48"/>
+      <c r="J19" s="20"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="3"/>
       <c r="C20" s="8"/>
-    </row>
-    <row r="21" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="66" t="s">
-        <v>11</v>
-      </c>
-      <c r="B21" s="67"/>
-      <c r="C21" s="67"/>
-      <c r="D21" s="67"/>
-      <c r="E21" s="67"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" s="68"/>
-      <c r="B22" s="69"/>
-      <c r="C22" s="69"/>
-      <c r="D22" s="69"/>
-      <c r="E22" s="69"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="68"/>
-      <c r="B23" s="69"/>
-      <c r="C23" s="69"/>
-      <c r="D23" s="69"/>
-      <c r="E23" s="69"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="68"/>
-      <c r="B24" s="69"/>
-      <c r="C24" s="69"/>
-      <c r="D24" s="69"/>
-      <c r="E24" s="69"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" s="3"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E20" s="26"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" s="3"/>
+      <c r="C21" s="8"/>
+    </row>
+    <row r="22" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="64" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22" s="65"/>
+      <c r="C22" s="65"/>
+      <c r="D22" s="65"/>
+      <c r="E22" s="65"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" s="66"/>
+      <c r="B23" s="67"/>
+      <c r="C23" s="67"/>
+      <c r="D23" s="67"/>
+      <c r="E23" s="67"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" s="66"/>
+      <c r="B24" s="67"/>
+      <c r="C24" s="67"/>
+      <c r="D24" s="67"/>
+      <c r="E24" s="67"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" s="66"/>
+      <c r="B25" s="67"/>
+      <c r="C25" s="67"/>
+      <c r="D25" s="67"/>
+      <c r="E25" s="67"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="3"/>
-      <c r="C26" s="8"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="3"/>
       <c r="C27" s="8"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="3"/>
       <c r="C28" s="8"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="3"/>
       <c r="C29" s="8"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="3"/>
       <c r="C30" s="8"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="3"/>
       <c r="C31" s="8"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C32" s="9"/>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" s="3"/>
+      <c r="C32" s="8"/>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C33" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A21:E24"/>
-    <mergeCell ref="A9:A18"/>
+    <mergeCell ref="A22:E25"/>
+    <mergeCell ref="A10:A19"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E3"/>
     <mergeCell ref="A4:E6"/>

</xml_diff>